<commit_message>
UPDATE CR2 y PR 2, PR 3
</commit_message>
<xml_diff>
--- a/documentation/Construccion y Evolucion/1. Solicitudes de cambio/CR 2.xlsx
+++ b/documentation/Construccion y Evolucion/1. Solicitudes de cambio/CR 2.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Proyectos\TraductorBraille\documentation\Construccion y Evolucion\1. Solicitudes de cambio\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USUARIO\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2C35738-3EDE-4811-BF95-A91B8E66B49B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98C66552-0152-45EE-A288-4AE138F75D1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11040" xr2:uid="{AAACD53E-982C-4521-B07F-7DC6290E23F5}"/>
+    <workbookView xWindow="-23148" yWindow="-2088" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{AAACD53E-982C-4521-B07F-7DC6290E23F5}"/>
   </bookViews>
   <sheets>
     <sheet name="CR Formato" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="49">
   <si>
     <t>CHANGE REQUEST</t>
   </si>
@@ -152,6 +152,29 @@
   </si>
   <si>
     <t>Victor Rodriguez</t>
+  </si>
+  <si>
+    <t>Brailingo - SoftTech</t>
+  </si>
+  <si>
+    <t>GUI</t>
+  </si>
+  <si>
+    <t>Aumento del tamaño de fuente en áreas específicas de traducción</t>
+  </si>
+  <si>
+    <t>1, Aumento Global del Tamaño de Fuente: Modificar el tamaño de fuente en todas las áreas de traducción de la interfaz de usuario para un tamaño de fuente uniforme.
+2. Configuración de Tamaño de Fuente Personalizable: Añadir una opción en la configuración de la aplicación que permita a los usuarios ajustar el tamaño de la fuente según sus preferencias.
+3. Aumento Selectivo del Tamaño de Fuente: Aumentar el tamaño de la fuente solo en los Text Area de traducción donde la legibilidad es más crítica.</t>
+  </si>
+  <si>
+    <t>8 horas</t>
+  </si>
+  <si>
+    <t>Uso mímino de 8 horas</t>
+  </si>
+  <si>
+    <t>Implementar la Alternativa de Aumento Global del Tamaño de Fuente para asegurar una mejora uniforme en la legibilidad de las áreas de traducción. Esta opción es la más directa y sencilla de aplicar, con un impacto mínimo en el cronograma del proyecto y sin requerir una personalización compleja.</t>
   </si>
 </sst>
 </file>
@@ -442,7 +465,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -476,6 +499,15 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="3" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -503,35 +535,49 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -868,7 +914,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67F84A08-0160-4953-9528-DB07A5F993CD}">
   <dimension ref="B1:H33"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="5.5703125" customWidth="1"/>
     <col min="3" max="3" width="36.42578125" bestFit="1" customWidth="1"/>
@@ -919,12 +965,12 @@
       <c r="C7" t="s">
         <v>3</v>
       </c>
-      <c r="D7" s="25" t="s">
+      <c r="D7" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="E7" s="25"/>
-      <c r="F7" s="25"/>
-      <c r="G7" s="25"/>
+      <c r="E7" s="28"/>
+      <c r="F7" s="28"/>
+      <c r="G7" s="28"/>
       <c r="H7" s="7"/>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
@@ -940,12 +986,12 @@
       <c r="C10" t="s">
         <v>4</v>
       </c>
-      <c r="D10" s="25" t="s">
+      <c r="D10" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="E10" s="25"/>
-      <c r="F10" s="25"/>
-      <c r="G10" s="25"/>
+      <c r="E10" s="28"/>
+      <c r="F10" s="28"/>
+      <c r="G10" s="28"/>
       <c r="H10" s="7"/>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.25">
@@ -957,12 +1003,12 @@
       <c r="C12" t="s">
         <v>5</v>
       </c>
-      <c r="D12" s="25" t="s">
+      <c r="D12" s="28" t="s">
         <v>39</v>
       </c>
-      <c r="E12" s="25"/>
-      <c r="F12" s="25"/>
-      <c r="G12" s="25"/>
+      <c r="E12" s="28"/>
+      <c r="F12" s="28"/>
+      <c r="G12" s="28"/>
       <c r="H12" s="7"/>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.25">
@@ -978,22 +1024,22 @@
     </row>
     <row r="15" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B15" s="4"/>
-      <c r="C15" s="26" t="s">
+      <c r="C15" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="D15" s="27"/>
-      <c r="E15" s="27"/>
-      <c r="F15" s="27"/>
-      <c r="G15" s="28"/>
+      <c r="D15" s="30"/>
+      <c r="E15" s="30"/>
+      <c r="F15" s="30"/>
+      <c r="G15" s="31"/>
       <c r="H15" s="7"/>
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B16" s="4"/>
-      <c r="C16" s="29"/>
-      <c r="D16" s="30"/>
-      <c r="E16" s="30"/>
-      <c r="F16" s="30"/>
-      <c r="G16" s="31"/>
+      <c r="C16" s="32"/>
+      <c r="D16" s="33"/>
+      <c r="E16" s="33"/>
+      <c r="F16" s="33"/>
+      <c r="G16" s="34"/>
       <c r="H16" s="7"/>
     </row>
     <row r="17" spans="2:8" x14ac:dyDescent="0.25">
@@ -1002,10 +1048,10 @@
     </row>
     <row r="18" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B18" s="4"/>
-      <c r="C18" s="32" t="s">
+      <c r="C18" s="35" t="s">
         <v>7</v>
       </c>
-      <c r="D18" s="33"/>
+      <c r="D18" s="36"/>
       <c r="E18" s="8" t="s">
         <v>8</v>
       </c>
@@ -1157,11 +1203,11 @@
     </row>
     <row r="32" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B32" s="4"/>
-      <c r="C32" s="34"/>
-      <c r="D32" s="35"/>
-      <c r="E32" s="35"/>
-      <c r="F32" s="35"/>
-      <c r="G32" s="36"/>
+      <c r="C32" s="25"/>
+      <c r="D32" s="26"/>
+      <c r="E32" s="26"/>
+      <c r="F32" s="26"/>
+      <c r="G32" s="27"/>
       <c r="H32" s="7"/>
     </row>
     <row r="33" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1189,7 +1235,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33198599-D7F8-440A-9813-85D60D291D95}">
   <dimension ref="B1:H34"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.5703125" customWidth="1"/>
     <col min="3" max="3" width="39" bestFit="1" customWidth="1"/>
@@ -1216,7 +1262,9 @@
       <c r="F3" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="17"/>
+      <c r="G3" s="17">
+        <v>2</v>
+      </c>
       <c r="H3" s="7"/>
     </row>
     <row r="4" spans="2:8" x14ac:dyDescent="0.25">
@@ -1224,7 +1272,9 @@
       <c r="F4" t="s">
         <v>26</v>
       </c>
-      <c r="G4" s="18"/>
+      <c r="G4" s="18">
+        <v>2</v>
+      </c>
       <c r="H4" s="7"/>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.25">
@@ -1232,7 +1282,9 @@
       <c r="F5" t="s">
         <v>27</v>
       </c>
-      <c r="G5" s="18"/>
+      <c r="G5" s="39">
+        <v>45517</v>
+      </c>
       <c r="H5" s="7"/>
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.25">
@@ -1244,7 +1296,9 @@
       <c r="C7" t="s">
         <v>3</v>
       </c>
-      <c r="D7" s="37"/>
+      <c r="D7" s="37" t="s">
+        <v>42</v>
+      </c>
       <c r="E7" s="37"/>
       <c r="F7" s="37"/>
       <c r="G7" s="37"/>
@@ -1267,47 +1321,49 @@
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B10" s="4"/>
-      <c r="C10" s="38"/>
-      <c r="D10" s="39"/>
-      <c r="E10" s="39"/>
-      <c r="F10" s="39"/>
-      <c r="G10" s="40"/>
+      <c r="C10" s="40" t="s">
+        <v>45</v>
+      </c>
+      <c r="D10" s="41"/>
+      <c r="E10" s="41"/>
+      <c r="F10" s="41"/>
+      <c r="G10" s="42"/>
       <c r="H10" s="7"/>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B11" s="4"/>
-      <c r="C11" s="38"/>
-      <c r="D11" s="39"/>
-      <c r="E11" s="39"/>
-      <c r="F11" s="39"/>
-      <c r="G11" s="40"/>
+      <c r="C11" s="43"/>
+      <c r="D11" s="41"/>
+      <c r="E11" s="41"/>
+      <c r="F11" s="41"/>
+      <c r="G11" s="42"/>
       <c r="H11" s="7"/>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B12" s="4"/>
-      <c r="C12" s="38"/>
-      <c r="D12" s="39"/>
-      <c r="E12" s="39"/>
-      <c r="F12" s="39"/>
-      <c r="G12" s="40"/>
+      <c r="C12" s="43"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="41"/>
+      <c r="F12" s="41"/>
+      <c r="G12" s="42"/>
       <c r="H12" s="7"/>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B13" s="4"/>
-      <c r="C13" s="38"/>
-      <c r="D13" s="39"/>
-      <c r="E13" s="39"/>
-      <c r="F13" s="39"/>
-      <c r="G13" s="40"/>
+      <c r="C13" s="43"/>
+      <c r="D13" s="41"/>
+      <c r="E13" s="41"/>
+      <c r="F13" s="41"/>
+      <c r="G13" s="42"/>
       <c r="H13" s="7"/>
     </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="4"/>
-      <c r="C14" s="41"/>
-      <c r="D14" s="42"/>
-      <c r="E14" s="42"/>
-      <c r="F14" s="42"/>
-      <c r="G14" s="43"/>
+      <c r="C14" s="44"/>
+      <c r="D14" s="45"/>
+      <c r="E14" s="45"/>
+      <c r="F14" s="45"/>
+      <c r="G14" s="46"/>
       <c r="H14" s="7"/>
     </row>
     <row r="15" spans="2:8" x14ac:dyDescent="0.25">
@@ -1326,54 +1382,58 @@
       <c r="C17" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="D17" s="34" t="s">
+      <c r="D17" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="E17" s="35"/>
-      <c r="F17" s="35"/>
-      <c r="G17" s="36"/>
+      <c r="E17" s="26"/>
+      <c r="F17" s="26"/>
+      <c r="G17" s="27"/>
       <c r="H17" s="7"/>
     </row>
     <row r="18" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B18" s="4"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="34"/>
-      <c r="E18" s="35"/>
-      <c r="F18" s="35"/>
-      <c r="G18" s="36"/>
+      <c r="C18" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="D18" s="25" t="s">
+        <v>44</v>
+      </c>
+      <c r="E18" s="26"/>
+      <c r="F18" s="26"/>
+      <c r="G18" s="27"/>
       <c r="H18" s="7"/>
     </row>
     <row r="19" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B19" s="4"/>
       <c r="C19" s="8"/>
-      <c r="D19" s="34"/>
-      <c r="E19" s="35"/>
-      <c r="F19" s="35"/>
-      <c r="G19" s="36"/>
+      <c r="D19" s="25"/>
+      <c r="E19" s="26"/>
+      <c r="F19" s="26"/>
+      <c r="G19" s="27"/>
       <c r="H19" s="7"/>
     </row>
     <row r="20" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B20" s="4"/>
       <c r="C20" s="8"/>
-      <c r="D20" s="34"/>
-      <c r="E20" s="35"/>
-      <c r="F20" s="35"/>
-      <c r="G20" s="36"/>
+      <c r="D20" s="25"/>
+      <c r="E20" s="26"/>
+      <c r="F20" s="26"/>
+      <c r="G20" s="27"/>
       <c r="H20" s="7"/>
     </row>
     <row r="21" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B21" s="4"/>
       <c r="C21" s="8"/>
-      <c r="D21" s="34"/>
-      <c r="E21" s="35"/>
-      <c r="F21" s="35"/>
-      <c r="G21" s="36"/>
+      <c r="D21" s="25"/>
+      <c r="E21" s="26"/>
+      <c r="F21" s="26"/>
+      <c r="G21" s="27"/>
       <c r="H21" s="7"/>
     </row>
     <row r="22" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B22" s="4"/>
-      <c r="F22" s="39"/>
-      <c r="G22" s="39"/>
+      <c r="F22" s="38"/>
+      <c r="G22" s="38"/>
       <c r="H22" s="7"/>
     </row>
     <row r="23" spans="2:8" x14ac:dyDescent="0.25">
@@ -1381,7 +1441,9 @@
       <c r="C23" t="s">
         <v>32</v>
       </c>
-      <c r="D23" s="17"/>
+      <c r="D23" s="17" t="s">
+        <v>46</v>
+      </c>
       <c r="H23" s="7"/>
     </row>
     <row r="24" spans="2:8" x14ac:dyDescent="0.25">
@@ -1400,7 +1462,9 @@
       <c r="C26" t="s">
         <v>34</v>
       </c>
-      <c r="D26" s="17"/>
+      <c r="D26" s="47" t="s">
+        <v>47</v>
+      </c>
       <c r="H26" s="7"/>
     </row>
     <row r="27" spans="2:8" x14ac:dyDescent="0.25">
@@ -1420,47 +1484,49 @@
     </row>
     <row r="29" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B29" s="4"/>
-      <c r="C29" s="38"/>
-      <c r="D29" s="39"/>
-      <c r="E29" s="39"/>
-      <c r="F29" s="39"/>
-      <c r="G29" s="40"/>
+      <c r="C29" s="40" t="s">
+        <v>48</v>
+      </c>
+      <c r="D29" s="48"/>
+      <c r="E29" s="48"/>
+      <c r="F29" s="48"/>
+      <c r="G29" s="49"/>
       <c r="H29" s="7"/>
     </row>
     <row r="30" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B30" s="4"/>
-      <c r="C30" s="38"/>
-      <c r="D30" s="39"/>
-      <c r="E30" s="39"/>
-      <c r="F30" s="39"/>
-      <c r="G30" s="40"/>
+      <c r="C30" s="40"/>
+      <c r="D30" s="48"/>
+      <c r="E30" s="48"/>
+      <c r="F30" s="48"/>
+      <c r="G30" s="49"/>
       <c r="H30" s="7"/>
     </row>
     <row r="31" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B31" s="4"/>
-      <c r="C31" s="38"/>
-      <c r="D31" s="39"/>
-      <c r="E31" s="39"/>
-      <c r="F31" s="39"/>
-      <c r="G31" s="40"/>
+      <c r="C31" s="40"/>
+      <c r="D31" s="48"/>
+      <c r="E31" s="48"/>
+      <c r="F31" s="48"/>
+      <c r="G31" s="49"/>
       <c r="H31" s="7"/>
     </row>
-    <row r="32" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:8" ht="3.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="4"/>
-      <c r="C32" s="38"/>
-      <c r="D32" s="39"/>
-      <c r="E32" s="39"/>
-      <c r="F32" s="39"/>
-      <c r="G32" s="40"/>
+      <c r="C32" s="40"/>
+      <c r="D32" s="48"/>
+      <c r="E32" s="48"/>
+      <c r="F32" s="48"/>
+      <c r="G32" s="49"/>
       <c r="H32" s="7"/>
     </row>
-    <row r="33" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:8" ht="3.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" s="4"/>
-      <c r="C33" s="41"/>
-      <c r="D33" s="42"/>
-      <c r="E33" s="42"/>
-      <c r="F33" s="42"/>
-      <c r="G33" s="43"/>
+      <c r="C33" s="50"/>
+      <c r="D33" s="51"/>
+      <c r="E33" s="51"/>
+      <c r="F33" s="51"/>
+      <c r="G33" s="52"/>
       <c r="H33" s="7"/>
     </row>
     <row r="34" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1497,15 +1563,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100B08EDF72D49EA44AB90F024D99D2B5E3" ma:contentTypeVersion="17" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="d6207507167e209dbfd27b884ee120ca">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="f7b1a7ea-1dd0-43bd-8f52-dd9459d0ec96" xmlns:ns4="56eae398-d265-4f71-b30c-62c529056c9f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7ebf290c66ec3e245dfaec660d84bc70" ns3:_="" ns4:_="">
     <xsd:import namespace="f7b1a7ea-1dd0-43bd-8f52-dd9459d0ec96"/>
@@ -1752,6 +1809,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{96BACB75-2D9E-4BF9-B15E-EA86EAB29BB3}">
   <ds:schemaRefs>
@@ -1770,14 +1836,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3BE880B-0D64-411C-BD75-74863A321A9B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A299727D-0257-4624-9B82-EEF7D307A1F7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1794,4 +1852,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3BE880B-0D64-411C-BD75-74863A321A9B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>